<commit_message>
feat: modelo com Horas digitavel (sem formula) e enxuto em 41 linhas
A coluna Horas (8) passa a ser preenchida a mao, ja que o lancamento
retroativo le e lanca essa coluna; antes ela trazia =K-J, que devolvia 0:00.
Modelo reduzido de 100 para 41 linhas; listas e validacoes preservadas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aquivo_modelo.xlsx
+++ b/aquivo_modelo.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programas VLF\ficha_tempo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55593E96-2DCB-498A-A195-F30CC179DEBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE49ED67-7F1B-4B96-A33B-264EE50F3F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookPassword="FC66" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10216" uniqueCount="10077">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10158" uniqueCount="10077">
   <si>
     <t>TipoF</t>
   </si>
@@ -30626,25 +30626,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P100"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.21875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.21875" customWidth="1"/>
+    <col min="3" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="20.109375" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" customWidth="1"/>
+    <col min="7" max="7" width="26.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="14" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5546875" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="21.109375" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="22.21875" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="24.6640625" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="7.77734375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" hidden="1" collapsed="1" x14ac:dyDescent="0.3">
@@ -30753,16 +30753,15 @@
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="E3" s="2"/>
       <c r="F3" s="3"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="5">
-        <f t="shared" ref="H3:H34" si="0">K3-J3</f>
-        <v>0</v>
-      </c>
+      <c r="H3" s="5"/>
       <c r="I3" s="5">
-        <f t="shared" ref="I3:I34" si="1">K3-J3</f>
+        <f t="shared" ref="I3:I34" si="0">K3-J3</f>
         <v>0</v>
       </c>
       <c r="J3" s="4"/>
@@ -30780,12 +30779,9 @@
       <c r="E4" s="2"/>
       <c r="F4" s="3"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="5">
+      <c r="H4" s="5"/>
+      <c r="I4" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I4" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J4" s="4"/>
@@ -30803,12 +30799,9 @@
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="5">
+      <c r="H5" s="5"/>
+      <c r="I5" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J5" s="4"/>
@@ -30826,12 +30819,9 @@
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="5">
+      <c r="H6" s="5"/>
+      <c r="I6" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J6" s="4"/>
@@ -30849,12 +30839,9 @@
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="5">
+      <c r="H7" s="5"/>
+      <c r="I7" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J7" s="4"/>
@@ -30872,12 +30859,9 @@
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="5">
+      <c r="H8" s="5"/>
+      <c r="I8" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J8" s="4"/>
@@ -30895,12 +30879,9 @@
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="5">
+      <c r="H9" s="5"/>
+      <c r="I9" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J9" s="4"/>
@@ -30918,12 +30899,9 @@
       <c r="E10" s="2"/>
       <c r="F10" s="3"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="5">
+      <c r="H10" s="5"/>
+      <c r="I10" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J10" s="4"/>
@@ -30941,12 +30919,9 @@
       <c r="E11" s="2"/>
       <c r="F11" s="3"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="5">
+      <c r="H11" s="5"/>
+      <c r="I11" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J11" s="4"/>
@@ -30964,12 +30939,9 @@
       <c r="E12" s="2"/>
       <c r="F12" s="3"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="5">
+      <c r="H12" s="5"/>
+      <c r="I12" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I12" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J12" s="4"/>
@@ -30987,12 +30959,9 @@
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
       <c r="G13" s="2"/>
-      <c r="H13" s="5">
+      <c r="H13" s="5"/>
+      <c r="I13" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J13" s="4"/>
@@ -31010,12 +30979,9 @@
       <c r="E14" s="2"/>
       <c r="F14" s="3"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="5">
+      <c r="H14" s="5"/>
+      <c r="I14" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J14" s="4"/>
@@ -31033,12 +30999,9 @@
       <c r="E15" s="2"/>
       <c r="F15" s="3"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="5">
+      <c r="H15" s="5"/>
+      <c r="I15" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J15" s="4"/>
@@ -31056,12 +31019,9 @@
       <c r="E16" s="2"/>
       <c r="F16" s="3"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="5">
+      <c r="H16" s="5"/>
+      <c r="I16" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J16" s="4"/>
@@ -31079,12 +31039,9 @@
       <c r="E17" s="2"/>
       <c r="F17" s="3"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="5">
+      <c r="H17" s="5"/>
+      <c r="I17" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I17" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J17" s="4"/>
@@ -31102,12 +31059,9 @@
       <c r="E18" s="2"/>
       <c r="F18" s="3"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="5">
+      <c r="H18" s="5"/>
+      <c r="I18" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I18" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J18" s="4"/>
@@ -31125,12 +31079,9 @@
       <c r="E19" s="2"/>
       <c r="F19" s="3"/>
       <c r="G19" s="2"/>
-      <c r="H19" s="5">
+      <c r="H19" s="5"/>
+      <c r="I19" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I19" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J19" s="4"/>
@@ -31148,12 +31099,9 @@
       <c r="E20" s="2"/>
       <c r="F20" s="3"/>
       <c r="G20" s="2"/>
-      <c r="H20" s="5">
+      <c r="H20" s="5"/>
+      <c r="I20" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J20" s="4"/>
@@ -31171,12 +31119,9 @@
       <c r="E21" s="2"/>
       <c r="F21" s="3"/>
       <c r="G21" s="2"/>
-      <c r="H21" s="5">
+      <c r="H21" s="5"/>
+      <c r="I21" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J21" s="4"/>
@@ -31194,12 +31139,9 @@
       <c r="E22" s="2"/>
       <c r="F22" s="3"/>
       <c r="G22" s="2"/>
-      <c r="H22" s="5">
+      <c r="H22" s="5"/>
+      <c r="I22" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I22" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J22" s="4"/>
@@ -31217,12 +31159,9 @@
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
       <c r="G23" s="2"/>
-      <c r="H23" s="5">
+      <c r="H23" s="5"/>
+      <c r="I23" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I23" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J23" s="4"/>
@@ -31240,12 +31179,9 @@
       <c r="E24" s="2"/>
       <c r="F24" s="3"/>
       <c r="G24" s="2"/>
-      <c r="H24" s="5">
+      <c r="H24" s="5"/>
+      <c r="I24" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I24" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J24" s="4"/>
@@ -31263,12 +31199,9 @@
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
       <c r="G25" s="2"/>
-      <c r="H25" s="5">
+      <c r="H25" s="5"/>
+      <c r="I25" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I25" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J25" s="4"/>
@@ -31286,12 +31219,9 @@
       <c r="E26" s="2"/>
       <c r="F26" s="3"/>
       <c r="G26" s="2"/>
-      <c r="H26" s="5">
+      <c r="H26" s="5"/>
+      <c r="I26" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I26" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J26" s="4"/>
@@ -31309,12 +31239,9 @@
       <c r="E27" s="2"/>
       <c r="F27" s="3"/>
       <c r="G27" s="2"/>
-      <c r="H27" s="5">
+      <c r="H27" s="5"/>
+      <c r="I27" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I27" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J27" s="4"/>
@@ -31332,12 +31259,9 @@
       <c r="E28" s="2"/>
       <c r="F28" s="3"/>
       <c r="G28" s="2"/>
-      <c r="H28" s="5">
+      <c r="H28" s="5"/>
+      <c r="I28" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I28" s="5">
-        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="J28" s="4"/>
@@ -31355,18 +31279,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="3"/>
       <c r="G29" s="2"/>
-      <c r="H29" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I29" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
+      <c r="H29" s="5"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -31378,18 +31291,7 @@
       <c r="E30" s="2"/>
       <c r="F30" s="3"/>
       <c r="G30" s="2"/>
-      <c r="H30" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I30" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
+      <c r="H30" s="5"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
@@ -31401,18 +31303,7 @@
       <c r="E31" s="2"/>
       <c r="F31" s="3"/>
       <c r="G31" s="2"/>
-      <c r="H31" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I31" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
+      <c r="H31" s="5"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -31424,20 +31315,9 @@
       <c r="E32" s="2"/>
       <c r="F32" s="3"/>
       <c r="G32" s="2"/>
-      <c r="H32" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I32" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -31447,20 +31327,9 @@
       <c r="E33" s="2"/>
       <c r="F33" s="3"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I33" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -31470,20 +31339,9 @@
       <c r="E34" s="2"/>
       <c r="F34" s="3"/>
       <c r="G34" s="2"/>
-      <c r="H34" s="5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I34" s="5">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="6"/>
-      <c r="M34" s="6"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -31493,20 +31351,9 @@
       <c r="E35" s="2"/>
       <c r="F35" s="3"/>
       <c r="G35" s="2"/>
-      <c r="H35" s="5">
-        <f t="shared" ref="H35:H66" si="2">K35-J35</f>
-        <v>0</v>
-      </c>
-      <c r="I35" s="5">
-        <f t="shared" ref="I35:I66" si="3">K35-J35</f>
-        <v>0</v>
-      </c>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -31516,20 +31363,9 @@
       <c r="E36" s="2"/>
       <c r="F36" s="3"/>
       <c r="G36" s="2"/>
-      <c r="H36" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I36" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="6"/>
-      <c r="M36" s="6"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>26</v>
       </c>
@@ -31539,20 +31375,9 @@
       <c r="E37" s="2"/>
       <c r="F37" s="3"/>
       <c r="G37" s="2"/>
-      <c r="H37" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I37" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="6"/>
-      <c r="M37" s="6"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -31562,20 +31387,9 @@
       <c r="E38" s="2"/>
       <c r="F38" s="3"/>
       <c r="G38" s="2"/>
-      <c r="H38" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I38" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="6"/>
-      <c r="M38" s="6"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H38" s="5"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>26</v>
       </c>
@@ -31585,20 +31399,9 @@
       <c r="E39" s="2"/>
       <c r="F39" s="3"/>
       <c r="G39" s="2"/>
-      <c r="H39" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I39" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>26</v>
       </c>
@@ -31608,20 +31411,9 @@
       <c r="E40" s="2"/>
       <c r="F40" s="3"/>
       <c r="G40" s="2"/>
-      <c r="H40" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I40" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="6"/>
-      <c r="M40" s="6"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>26</v>
       </c>
@@ -31631,1375 +31423,7 @@
       <c r="E41" s="2"/>
       <c r="F41" s="3"/>
       <c r="G41" s="2"/>
-      <c r="H41" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I41" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="6"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>26</v>
-      </c>
-      <c r="B42" s="1"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I42" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="6"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>26</v>
-      </c>
-      <c r="B43" s="1"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="3"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I43" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="6"/>
-      <c r="M43" s="6"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>26</v>
-      </c>
-      <c r="B44" s="1"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="3"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I44" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="6"/>
-      <c r="M44" s="6"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" s="1"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="3"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I45" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="6"/>
-      <c r="M45" s="6"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>26</v>
-      </c>
-      <c r="B46" s="1"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I46" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J46" s="4"/>
-      <c r="K46" s="4"/>
-      <c r="L46" s="6"/>
-      <c r="M46" s="6"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>26</v>
-      </c>
-      <c r="B47" s="1"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I47" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="6"/>
-      <c r="M47" s="6"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>26</v>
-      </c>
-      <c r="B48" s="1"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="2"/>
-      <c r="H48" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I48" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>26</v>
-      </c>
-      <c r="B49" s="1"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="2"/>
-      <c r="H49" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I49" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J49" s="4"/>
-      <c r="K49" s="4"/>
-      <c r="L49" s="6"/>
-      <c r="M49" s="6"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>26</v>
-      </c>
-      <c r="B50" s="1"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="2"/>
-      <c r="H50" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I50" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="6"/>
-      <c r="M50" s="6"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>26</v>
-      </c>
-      <c r="B51" s="1"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="2"/>
-      <c r="H51" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I51" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="6"/>
-      <c r="M51" s="6"/>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>26</v>
-      </c>
-      <c r="B52" s="1"/>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="3"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I52" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J52" s="4"/>
-      <c r="K52" s="4"/>
-      <c r="L52" s="6"/>
-      <c r="M52" s="6"/>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>26</v>
-      </c>
-      <c r="B53" s="1"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="3"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I53" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J53" s="4"/>
-      <c r="K53" s="4"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="6"/>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>26</v>
-      </c>
-      <c r="B54" s="1"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="2"/>
-      <c r="H54" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I54" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6"/>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>26</v>
-      </c>
-      <c r="B55" s="1"/>
-      <c r="C55" s="2"/>
-      <c r="D55" s="2"/>
-      <c r="E55" s="2"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="2"/>
-      <c r="H55" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I55" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J55" s="4"/>
-      <c r="K55" s="4"/>
-      <c r="L55" s="6"/>
-      <c r="M55" s="6"/>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>26</v>
-      </c>
-      <c r="B56" s="1"/>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="3"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I56" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
-      <c r="L56" s="6"/>
-      <c r="M56" s="6"/>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B57" s="1"/>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="2"/>
-      <c r="H57" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I57" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="L57" s="6"/>
-      <c r="M57" s="6"/>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>26</v>
-      </c>
-      <c r="B58" s="1"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="2"/>
-      <c r="H58" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I58" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="6"/>
-      <c r="M58" s="6"/>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>26</v>
-      </c>
-      <c r="B59" s="1"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="3"/>
-      <c r="G59" s="2"/>
-      <c r="H59" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I59" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J59" s="4"/>
-      <c r="K59" s="4"/>
-      <c r="L59" s="6"/>
-      <c r="M59" s="6"/>
-    </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>26</v>
-      </c>
-      <c r="B60" s="1"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="3"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I60" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J60" s="4"/>
-      <c r="K60" s="4"/>
-      <c r="L60" s="6"/>
-      <c r="M60" s="6"/>
-    </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>26</v>
-      </c>
-      <c r="B61" s="1"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="3"/>
-      <c r="G61" s="2"/>
-      <c r="H61" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I61" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J61" s="4"/>
-      <c r="K61" s="4"/>
-      <c r="L61" s="6"/>
-      <c r="M61" s="6"/>
-    </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>26</v>
-      </c>
-      <c r="B62" s="1"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I62" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J62" s="4"/>
-      <c r="K62" s="4"/>
-      <c r="L62" s="6"/>
-      <c r="M62" s="6"/>
-    </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>26</v>
-      </c>
-      <c r="B63" s="1"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="3"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I63" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="6"/>
-      <c r="M63" s="6"/>
-    </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>26</v>
-      </c>
-      <c r="B64" s="1"/>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I64" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="6"/>
-      <c r="M64" s="6"/>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>26</v>
-      </c>
-      <c r="B65" s="1"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="3"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I65" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J65" s="4"/>
-      <c r="K65" s="4"/>
-      <c r="L65" s="6"/>
-      <c r="M65" s="6"/>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>26</v>
-      </c>
-      <c r="B66" s="1"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="3"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="5">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I66" s="5">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J66" s="4"/>
-      <c r="K66" s="4"/>
-      <c r="L66" s="6"/>
-      <c r="M66" s="6"/>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>26</v>
-      </c>
-      <c r="B67" s="1"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="E67" s="2"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="2"/>
-      <c r="H67" s="5">
-        <f t="shared" ref="H67:H100" si="4">K67-J67</f>
-        <v>0</v>
-      </c>
-      <c r="I67" s="5">
-        <f t="shared" ref="I67:I98" si="5">K67-J67</f>
-        <v>0</v>
-      </c>
-      <c r="J67" s="4"/>
-      <c r="K67" s="4"/>
-      <c r="L67" s="6"/>
-      <c r="M67" s="6"/>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>26</v>
-      </c>
-      <c r="B68" s="1"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="3"/>
-      <c r="G68" s="2"/>
-      <c r="H68" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I68" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J68" s="4"/>
-      <c r="K68" s="4"/>
-      <c r="L68" s="6"/>
-      <c r="M68" s="6"/>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>26</v>
-      </c>
-      <c r="B69" s="1"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="3"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I69" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J69" s="4"/>
-      <c r="K69" s="4"/>
-      <c r="L69" s="6"/>
-      <c r="M69" s="6"/>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>26</v>
-      </c>
-      <c r="B70" s="1"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="E70" s="2"/>
-      <c r="F70" s="3"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I70" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J70" s="4"/>
-      <c r="K70" s="4"/>
-      <c r="L70" s="6"/>
-      <c r="M70" s="6"/>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>26</v>
-      </c>
-      <c r="B71" s="1"/>
-      <c r="C71" s="2"/>
-      <c r="D71" s="2"/>
-      <c r="E71" s="2"/>
-      <c r="F71" s="3"/>
-      <c r="G71" s="2"/>
-      <c r="H71" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I71" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J71" s="4"/>
-      <c r="K71" s="4"/>
-      <c r="L71" s="6"/>
-      <c r="M71" s="6"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>26</v>
-      </c>
-      <c r="B72" s="1"/>
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="E72" s="2"/>
-      <c r="F72" s="3"/>
-      <c r="G72" s="2"/>
-      <c r="H72" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I72" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J72" s="4"/>
-      <c r="K72" s="4"/>
-      <c r="L72" s="6"/>
-      <c r="M72" s="6"/>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>26</v>
-      </c>
-      <c r="B73" s="1"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I73" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J73" s="4"/>
-      <c r="K73" s="4"/>
-      <c r="L73" s="6"/>
-      <c r="M73" s="6"/>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>26</v>
-      </c>
-      <c r="B74" s="1"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I74" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J74" s="4"/>
-      <c r="K74" s="4"/>
-      <c r="L74" s="6"/>
-      <c r="M74" s="6"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>26</v>
-      </c>
-      <c r="B75" s="1"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I75" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J75" s="4"/>
-      <c r="K75" s="4"/>
-      <c r="L75" s="6"/>
-      <c r="M75" s="6"/>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>26</v>
-      </c>
-      <c r="B76" s="1"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I76" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J76" s="4"/>
-      <c r="K76" s="4"/>
-      <c r="L76" s="6"/>
-      <c r="M76" s="6"/>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>26</v>
-      </c>
-      <c r="B77" s="1"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="3"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I77" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J77" s="4"/>
-      <c r="K77" s="4"/>
-      <c r="L77" s="6"/>
-      <c r="M77" s="6"/>
-    </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>26</v>
-      </c>
-      <c r="B78" s="1"/>
-      <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="3"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I78" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J78" s="4"/>
-      <c r="K78" s="4"/>
-      <c r="L78" s="6"/>
-      <c r="M78" s="6"/>
-    </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>26</v>
-      </c>
-      <c r="B79" s="1"/>
-      <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="3"/>
-      <c r="G79" s="2"/>
-      <c r="H79" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I79" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J79" s="4"/>
-      <c r="K79" s="4"/>
-      <c r="L79" s="6"/>
-      <c r="M79" s="6"/>
-    </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>26</v>
-      </c>
-      <c r="B80" s="1"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="F80" s="3"/>
-      <c r="G80" s="2"/>
-      <c r="H80" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I80" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J80" s="4"/>
-      <c r="K80" s="4"/>
-      <c r="L80" s="6"/>
-      <c r="M80" s="6"/>
-    </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>26</v>
-      </c>
-      <c r="B81" s="1"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="3"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I81" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J81" s="4"/>
-      <c r="K81" s="4"/>
-      <c r="L81" s="6"/>
-      <c r="M81" s="6"/>
-    </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>26</v>
-      </c>
-      <c r="B82" s="1"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="3"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I82" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J82" s="4"/>
-      <c r="K82" s="4"/>
-      <c r="L82" s="6"/>
-      <c r="M82" s="6"/>
-    </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>26</v>
-      </c>
-      <c r="B83" s="1"/>
-      <c r="C83" s="2"/>
-      <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
-      <c r="F83" s="3"/>
-      <c r="G83" s="2"/>
-      <c r="H83" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I83" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J83" s="4"/>
-      <c r="K83" s="4"/>
-      <c r="L83" s="6"/>
-      <c r="M83" s="6"/>
-    </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>26</v>
-      </c>
-      <c r="B84" s="1"/>
-      <c r="C84" s="2"/>
-      <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="2"/>
-      <c r="H84" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I84" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J84" s="4"/>
-      <c r="K84" s="4"/>
-      <c r="L84" s="6"/>
-      <c r="M84" s="6"/>
-    </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>26</v>
-      </c>
-      <c r="B85" s="1"/>
-      <c r="C85" s="2"/>
-      <c r="D85" s="2"/>
-      <c r="E85" s="2"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="2"/>
-      <c r="H85" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I85" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J85" s="4"/>
-      <c r="K85" s="4"/>
-      <c r="L85" s="6"/>
-      <c r="M85" s="6"/>
-    </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
-        <v>26</v>
-      </c>
-      <c r="B86" s="1"/>
-      <c r="C86" s="2"/>
-      <c r="D86" s="2"/>
-      <c r="E86" s="2"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="2"/>
-      <c r="H86" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I86" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J86" s="4"/>
-      <c r="K86" s="4"/>
-      <c r="L86" s="6"/>
-      <c r="M86" s="6"/>
-    </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
-        <v>26</v>
-      </c>
-      <c r="B87" s="1"/>
-      <c r="C87" s="2"/>
-      <c r="D87" s="2"/>
-      <c r="E87" s="2"/>
-      <c r="F87" s="3"/>
-      <c r="G87" s="2"/>
-      <c r="H87" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I87" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J87" s="4"/>
-      <c r="K87" s="4"/>
-      <c r="L87" s="6"/>
-      <c r="M87" s="6"/>
-    </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
-        <v>26</v>
-      </c>
-      <c r="B88" s="1"/>
-      <c r="C88" s="2"/>
-      <c r="D88" s="2"/>
-      <c r="E88" s="2"/>
-      <c r="F88" s="3"/>
-      <c r="G88" s="2"/>
-      <c r="H88" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I88" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J88" s="4"/>
-      <c r="K88" s="4"/>
-      <c r="L88" s="6"/>
-      <c r="M88" s="6"/>
-    </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A89" t="s">
-        <v>26</v>
-      </c>
-      <c r="B89" s="1"/>
-      <c r="C89" s="2"/>
-      <c r="D89" s="2"/>
-      <c r="E89" s="2"/>
-      <c r="F89" s="3"/>
-      <c r="G89" s="2"/>
-      <c r="H89" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I89" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J89" s="4"/>
-      <c r="K89" s="4"/>
-      <c r="L89" s="6"/>
-      <c r="M89" s="6"/>
-    </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A90" t="s">
-        <v>26</v>
-      </c>
-      <c r="B90" s="1"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
-      <c r="F90" s="3"/>
-      <c r="G90" s="2"/>
-      <c r="H90" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I90" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J90" s="4"/>
-      <c r="K90" s="4"/>
-      <c r="L90" s="6"/>
-      <c r="M90" s="6"/>
-    </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A91" t="s">
-        <v>26</v>
-      </c>
-      <c r="B91" s="1"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="3"/>
-      <c r="G91" s="2"/>
-      <c r="H91" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I91" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J91" s="4"/>
-      <c r="K91" s="4"/>
-      <c r="L91" s="6"/>
-      <c r="M91" s="6"/>
-    </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>26</v>
-      </c>
-      <c r="B92" s="1"/>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="3"/>
-      <c r="G92" s="2"/>
-      <c r="H92" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I92" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J92" s="4"/>
-      <c r="K92" s="4"/>
-      <c r="L92" s="6"/>
-      <c r="M92" s="6"/>
-    </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A93" t="s">
-        <v>26</v>
-      </c>
-      <c r="B93" s="1"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="3"/>
-      <c r="G93" s="2"/>
-      <c r="H93" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I93" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J93" s="4"/>
-      <c r="K93" s="4"/>
-      <c r="L93" s="6"/>
-      <c r="M93" s="6"/>
-    </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
-        <v>26</v>
-      </c>
-      <c r="B94" s="1"/>
-      <c r="C94" s="2"/>
-      <c r="D94" s="2"/>
-      <c r="E94" s="2"/>
-      <c r="F94" s="3"/>
-      <c r="G94" s="2"/>
-      <c r="H94" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I94" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J94" s="4"/>
-      <c r="K94" s="4"/>
-      <c r="L94" s="6"/>
-      <c r="M94" s="6"/>
-    </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A95" t="s">
-        <v>26</v>
-      </c>
-      <c r="B95" s="1"/>
-      <c r="C95" s="2"/>
-      <c r="D95" s="2"/>
-      <c r="E95" s="2"/>
-      <c r="F95" s="3"/>
-      <c r="G95" s="2"/>
-      <c r="H95" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I95" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J95" s="4"/>
-      <c r="K95" s="4"/>
-      <c r="L95" s="6"/>
-      <c r="M95" s="6"/>
-    </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>26</v>
-      </c>
-      <c r="B96" s="1"/>
-      <c r="C96" s="2"/>
-      <c r="D96" s="2"/>
-      <c r="E96" s="2"/>
-      <c r="F96" s="3"/>
-      <c r="G96" s="2"/>
-      <c r="H96" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I96" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J96" s="4"/>
-      <c r="K96" s="4"/>
-      <c r="L96" s="6"/>
-      <c r="M96" s="6"/>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>26</v>
-      </c>
-      <c r="B97" s="1"/>
-      <c r="C97" s="2"/>
-      <c r="D97" s="2"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="3"/>
-      <c r="G97" s="2"/>
-      <c r="H97" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I97" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J97" s="4"/>
-      <c r="K97" s="4"/>
-      <c r="L97" s="6"/>
-      <c r="M97" s="6"/>
-    </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>26</v>
-      </c>
-      <c r="B98" s="1"/>
-      <c r="C98" s="2"/>
-      <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
-      <c r="F98" s="3"/>
-      <c r="G98" s="2"/>
-      <c r="H98" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I98" s="5">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J98" s="4"/>
-      <c r="K98" s="4"/>
-      <c r="L98" s="6"/>
-      <c r="M98" s="6"/>
-    </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>26</v>
-      </c>
-      <c r="B99" s="1"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-      <c r="F99" s="3"/>
-      <c r="G99" s="2"/>
-      <c r="H99" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I99" s="5">
-        <f t="shared" ref="I99:I130" si="6">K99-J99</f>
-        <v>0</v>
-      </c>
-      <c r="J99" s="4"/>
-      <c r="K99" s="4"/>
-      <c r="L99" s="6"/>
-      <c r="M99" s="6"/>
-    </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
-        <v>26</v>
-      </c>
-      <c r="B100" s="1"/>
-      <c r="C100" s="2"/>
-      <c r="D100" s="2"/>
-      <c r="E100" s="2"/>
-      <c r="F100" s="3"/>
-      <c r="G100" s="2"/>
-      <c r="H100" s="5">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I100" s="5">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="J100" s="4"/>
-      <c r="K100" s="4"/>
-      <c r="L100" s="6"/>
-      <c r="M100" s="6"/>
+      <c r="H41" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -33010,43 +31434,43 @@
           <x14:formula1>
             <xm:f>TipoF!$A$1:A2</xm:f>
           </x14:formula1>
-          <xm:sqref>A3:A100</xm:sqref>
+          <xm:sqref>A3:A41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Advogado" prompt="Advogado" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Advogado!$A$1:A85</xm:f>
           </x14:formula1>
-          <xm:sqref>C3:C100</xm:sqref>
+          <xm:sqref>C3:C41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Tipo de Serviço" prompt="Tipo de Serviço" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Tipo!$A$1:A3</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D100</xm:sqref>
+          <xm:sqref>D3:D41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Cliente" prompt="Cliente" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>Cliente!$A$1:A1784</xm:f>
           </x14:formula1>
-          <xm:sqref>E3:E100</xm:sqref>
+          <xm:sqref>E3:E41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" operator="lessThan" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Pasta" prompt="Pasta" xr:uid="{00000000-0002-0000-0000-000004000000}">
           <x14:formula1>
             <xm:f>Pasta!$A$1:A7977</xm:f>
           </x14:formula1>
-          <xm:sqref>F3:F100</xm:sqref>
+          <xm:sqref>F3:F41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Parte Representada" prompt="Parte Representada" xr:uid="{00000000-0002-0000-0000-000005000000}">
           <x14:formula1>
             <xm:f>PRConta!$A$1:A234</xm:f>
           </x14:formula1>
-          <xm:sqref>N3:N100</xm:sqref>
+          <xm:sqref>N3:N28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Input error" error="Value is not in list." promptTitle="Unidade" prompt="Unidade" xr:uid="{00000000-0002-0000-0000-000006000000}">
           <x14:formula1>
             <xm:f>Unidade!$A$1:A1</xm:f>
           </x14:formula1>
-          <xm:sqref>P3:P100</xm:sqref>
+          <xm:sqref>P3:P28</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
feat: atualiza a relacao de advogados do modelo
Aba Advogado substituida pela nova relacao (85 nomes: 3 entram, 3 saem).
Demais abas e validacoes do modelo inalteradas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/aquivo_modelo.xlsx
+++ b/aquivo_modelo.xlsx
@@ -31505,428 +31505,598 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>29</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Acompanhamento de Processos</t>
+        </is>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>30</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Adriano Rodrigues Santos</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>31</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aline Piteres Porto</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>32</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Amanda Jardim de Souza</t>
+        </is>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>33</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ana Cláudia V. Veríssimo</t>
+        </is>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>34</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anderson Soares Freire</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>35</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">André Matos de Almeida Oliveira</t>
+        </is>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>36</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Anna Júlia Silva Costa</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>37</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Arthur Paredes Brandão</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>38</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Christian Sahb Batista Lopes</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>39</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONTROLADORIA DVB</t>
+        </is>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>40</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONTROLADORIA LMW</t>
+        </is>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>41</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONTROLADORIA RF/MB</t>
+        </is>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>42</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CORRESPONDENTE</t>
+        </is>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>43</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Daniel Rivoredo Vilas Boas (DVB)</t>
+        </is>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>44</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Danilo César Rezende Reis Gonçalves</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>45</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Débora Melillo de Almeida Gomes</t>
+        </is>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>46</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Eduardo Metzker Fernandes</t>
+        </is>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>47</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estefânia Mota Vieira Fonseca</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>48</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EXTERNO</t>
+        </is>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>49</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fabiola Santos Silva</t>
+        </is>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>50</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fernanda de Figueiredo Gomes</t>
+        </is>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>51</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fernanda Marra Vidigal</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>52</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gabrielle Aparecida de Melo Aleluia</t>
+        </is>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>53</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Géssica Karoline Morais Ribeiro</t>
+        </is>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>54</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giovanna Ramos Villegas</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>55</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Giovanni Augusto do Carmo Rodrigues</t>
+        </is>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>56</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gleiciane Soares Silva</t>
+        </is>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>57</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guilherme Leles Vieira</t>
+        </is>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>58</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Henrique Cabral Leão</t>
+        </is>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>59</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Henrique Coimbra Figueiredo</t>
+        </is>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>60</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Henrique Costa Abrantes</t>
+        </is>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>61</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hudson Ferrari Reis</t>
+        </is>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>62</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Isabelle Kelly Coelho Felix</t>
+        </is>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>63</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jéssica Nayra Santos Chebile</t>
+        </is>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>64</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joaquim Alvarenga Andrade e Silva</t>
+        </is>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>65</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Julia Fonseca Salomão</t>
+        </is>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>66</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Katryn de Souza Rocha</t>
+        </is>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>67</v>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kênia Késsia Dias de Sousa</t>
+        </is>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>68</v>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larissa Santos Morais</t>
+        </is>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>69</v>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leila Francisca Mendes Ferreira</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>70</v>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leilaine de Melo Vieira Queiroz</t>
+        </is>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>71</v>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leonardo Alves Corrêa</t>
+        </is>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A44" t="s">
-        <v>72</v>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leonardo Martins Wykrota</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>73</v>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lívia Mangelli Ferraz</t>
+        </is>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>74</v>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lorena Carvalho Lara</t>
+        </is>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>75</v>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lorena Machado de Oliveira</t>
+        </is>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>76</v>
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Oliveira Pignataro Claudino</t>
+        </is>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" t="s">
-        <v>77</v>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lucas Santos Auer</t>
+        </is>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>78</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luise Betzel Figueiredo</t>
+        </is>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>79</v>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcela Sousa Camargos</t>
+        </is>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>80</v>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Marcelo Baltar Bastos</t>
+        </is>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>81</v>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maria da Conceição Duque</t>
+        </is>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" t="s">
-        <v>82</v>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maria Eduarda Boson</t>
+        </is>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>83</v>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maria Eduarda Camargo de Oliveira</t>
+        </is>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>84</v>
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maria Tereza Fonseca Dias (MTF)</t>
+        </is>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>85</v>
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maria Victória Ferreira Werneck</t>
+        </is>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>86</v>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mariana dos Santos e Silva</t>
+        </is>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>87</v>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mariana Gomes Ramos</t>
+        </is>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>88</v>
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Matheus Emiliano de Almeida</t>
+        </is>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>89</v>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nayara Padilha Palma</t>
+        </is>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" t="s">
-        <v>90</v>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Osvaldo Braga Tolentino Veloso</t>
+        </is>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" t="s">
-        <v>91</v>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paula Martino Cota Dias</t>
+        </is>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" t="s">
-        <v>92</v>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paulo Vitor Ângelo Teixeira Sousa</t>
+        </is>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" t="s">
-        <v>93</v>
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedro Ernesto Gomes Rocha</t>
+        </is>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" t="s">
-        <v>94</v>
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PROTOCOLO ELETRÔNICO</t>
+        </is>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" t="s">
-        <v>95</v>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rafael de Albuquerque Rodrigues Queiroz</t>
+        </is>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>96</v>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rafhael Frattari Bonito</t>
+        </is>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A69" t="s">
-        <v>97</v>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samuel Augusto Cordeiro Gonçalves</t>
+        </is>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A70" t="s">
-        <v>98</v>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Samuel Francisco de Oliveira Pinto</t>
+        </is>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>99</v>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Silvana de Oliveira Medeiros</t>
+        </is>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A72" t="s">
-        <v>100</v>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sofia Garbarino Nogueira</t>
+        </is>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A73" t="s">
-        <v>101</v>
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suporte de TI - Suprema</t>
+        </is>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A74" t="s">
-        <v>102</v>
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Talita Ferreira de Brito dos Reis</t>
+        </is>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A75" t="s">
-        <v>103</v>
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Thales Vasconcelos Assunção Batista</t>
+        </is>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>104</v>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TWT Suporte</t>
+        </is>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>105</v>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vanessa Aparecida Alves</t>
+        </is>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
-        <v>106</v>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Victor Matheus Moreira da Silva Neves</t>
+        </is>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>107</v>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Victoria Nascimento Portela</t>
+        </is>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>108</v>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinícius Augustus de Vasconcelos Rezende Alves</t>
+        </is>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>109</v>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vinícius Ferreira de Jesus</t>
+        </is>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
-        <v>110</v>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wallison Sérgio Martins dos Passos</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
-        <v>111</v>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Walter de Souza Neto</t>
+        </is>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
-        <v>112</v>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wander Junio de Almeida</t>
+        </is>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
-        <v>113</v>
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yuri Brizon Reis</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>